<commit_message>
Update generated types and docs
</commit_message>
<xml_diff>
--- a/docs/financial-model-3yr.xlsx
+++ b/docs/financial-model-3yr.xlsx
@@ -599,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -657,7 +657,7 @@
       </c>
       <c r="D4" s="7">
         <f>B4*C4</f>
-        <v/>
+        <v>59.5</v>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
@@ -679,7 +679,7 @@
       </c>
       <c r="D5" s="7">
         <f>B5*C5</f>
-        <v/>
+        <v>21</v>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
@@ -701,7 +701,7 @@
       </c>
       <c r="D6" s="7">
         <f>B6*C6</f>
-        <v/>
+        <v>84</v>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
@@ -717,7 +717,7 @@
       </c>
       <c r="D7" s="9">
         <f>SUM(D4:D6)</f>
-        <v/>
+        <v>164.5</v>
       </c>
     </row>
     <row r="8">
@@ -748,7 +748,7 @@
       </c>
       <c r="D10" s="11">
         <f>D7+D8+D9</f>
-        <v/>
+        <v>221.5</v>
       </c>
     </row>
     <row r="12">
@@ -774,7 +774,7 @@
       </c>
       <c r="B13" s="13">
         <f>D10*B12</f>
-        <v/>
+        <v>38762.5</v>
       </c>
     </row>
     <row r="15">
@@ -785,7 +785,7 @@
       </c>
       <c r="B15" s="14">
         <f>D10*125</f>
-        <v/>
+        <v>27687.5</v>
       </c>
     </row>
     <row r="16">
@@ -796,13 +796,161 @@
       </c>
       <c r="B16" s="14">
         <f>D10*225</f>
-        <v/>
+        <v>49837.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Method: hours/day are estimates (blue — adjust them); commit counts and active days are measured facts from git.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>BEFORE 2026 — two earlier versions across ~10 years. Rows below are placeholder guesses: EDIT B and C to your memory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Era</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Years active</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Avg hrs/week</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Version 1 — first build (name/dates: edit)</t>
+        </is>
+      </c>
+      <c r="B22">
+        <v>3</v>
+      </c>
+      <c r="C22">
+        <v>3</v>
+      </c>
+      <c r="D22">
+        <f>B22*C22*52</f>
+        <v>468</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>guess — edit</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Version 2 — second build (name/dates: edit)</t>
+        </is>
+      </c>
+      <c r="B23">
+        <v>2</v>
+      </c>
+      <c r="C23">
+        <v>4</v>
+      </c>
+      <c r="D23">
+        <f>B23*C23*52</f>
+        <v>416</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>guess — edit</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Prior hours subtotal</t>
+        </is>
+      </c>
+      <c r="D24">
+        <f>SUM(D22:D23)</f>
+        <v>884</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Rate for prior work, $/hr</t>
+        </is>
+      </c>
+      <c r="B25">
+        <v>175</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>same market rate as current work</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Carry-forward factor</t>
+        </is>
+      </c>
+      <c r="B26">
+        <v>0.35</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>share of the old work still serving today: brand, audience, content, lessons. Edit 0–1</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Prior versions value</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>D24*B25*B26</f>
+        <v>54145</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL sweat equity (2026 work + prior carry-forward)</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>B13+B27</f>
+        <v>92907.5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Second lens: replacement cost — what an agency would charge to rebuild what existed Jan 1, 2026 (a comparable community app: $50k–150k). In investor talk, use whichever lens is higher and name the method.</t>
         </is>
       </c>
     </row>
@@ -929,11 +1077,11 @@
         </is>
       </c>
       <c r="B9" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>POLICY TOGGLE — decides breakeven; see README</t>
+          <t>DECIDED 2026-09-08: payer covers processing at checkout</t>
         </is>
       </c>
     </row>
@@ -1325,15 +1473,15 @@
       </c>
       <c r="B13" s="14">
         <f>B4*Inputs!$B$3*12</f>
-        <v/>
+        <v>18000</v>
       </c>
       <c r="C13" s="14">
         <f>C4*Inputs!$B$3*12</f>
-        <v/>
+        <v>48000</v>
       </c>
       <c r="D13" s="14">
         <f>D4*Inputs!$B$3*12</f>
-        <v/>
+        <v>108000</v>
       </c>
     </row>
     <row r="14">
@@ -1344,15 +1492,15 @@
       </c>
       <c r="B14" s="14">
         <f>B4*B6</f>
-        <v/>
+        <v>9000</v>
       </c>
       <c r="C14" s="14">
         <f>C4*C6</f>
-        <v/>
+        <v>32000</v>
       </c>
       <c r="D14" s="14">
         <f>D4*D6</f>
-        <v/>
+        <v>90000</v>
       </c>
     </row>
     <row r="15">
@@ -1363,15 +1511,15 @@
       </c>
       <c r="B15" s="13">
         <f>B13+B14</f>
-        <v/>
+        <v>27000</v>
       </c>
       <c r="C15" s="13">
         <f>C13+C14</f>
-        <v/>
+        <v>80000</v>
       </c>
       <c r="D15" s="13">
         <f>D13+D14</f>
-        <v/>
+        <v>198000</v>
       </c>
     </row>
     <row r="16">
@@ -1382,15 +1530,15 @@
       </c>
       <c r="B16" s="14">
         <f>B15*Inputs!$B$4</f>
-        <v/>
+        <v>2700</v>
       </c>
       <c r="C16" s="14">
         <f>C15*Inputs!$B$4</f>
-        <v/>
+        <v>8000</v>
       </c>
       <c r="D16" s="14">
         <f>D15*Inputs!$B$4</f>
-        <v/>
+        <v>19800</v>
       </c>
     </row>
     <row r="17">
@@ -1401,15 +1549,15 @@
       </c>
       <c r="B17" s="14">
         <f>Inputs!$B$9*((B13*(Inputs!$B$5+Inputs!$B$7))+(B4*12*Inputs!$B$6)+(B14*(Inputs!$B$5+Inputs!$B$7))+(B14/Inputs!$B$8*Inputs!$B$6))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C17" s="14">
         <f>Inputs!$B$9*((C13*(Inputs!$B$5+Inputs!$B$7))+(C4*12*Inputs!$B$6)+(C14*(Inputs!$B$5+Inputs!$B$7))+(C14/Inputs!$B$8*Inputs!$B$6))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D17" s="14">
         <f>Inputs!$B$9*((D13*(Inputs!$B$5+Inputs!$B$7))+(D4*12*Inputs!$B$6)+(D14*(Inputs!$B$5+Inputs!$B$7))+(D14/Inputs!$B$8*Inputs!$B$6))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1420,15 +1568,15 @@
       </c>
       <c r="B18" s="13">
         <f>B16-B17</f>
-        <v/>
+        <v>2700</v>
       </c>
       <c r="C18" s="13">
         <f>C16-C17</f>
-        <v/>
+        <v>8000</v>
       </c>
       <c r="D18" s="13">
         <f>D16-D17</f>
-        <v/>
+        <v>19800</v>
       </c>
     </row>
     <row r="20">
@@ -1462,15 +1610,15 @@
       </c>
       <c r="B22" s="14">
         <f>B4*Inputs!$B$10*12/1000*Inputs!$B$11</f>
-        <v/>
+        <v>12.6</v>
       </c>
       <c r="C22" s="14">
         <f>C4*Inputs!$B$10*12/1000*Inputs!$B$11</f>
-        <v/>
+        <v>33.6</v>
       </c>
       <c r="D22" s="14">
         <f>D4*Inputs!$B$10*12/1000*Inputs!$B$11</f>
-        <v/>
+        <v>75.6</v>
       </c>
     </row>
     <row r="23">
@@ -1481,15 +1629,15 @@
       </c>
       <c r="B23" s="14">
         <f>B7*Inputs!$B$12*Inputs!$B$13</f>
-        <v/>
+        <v>52.47</v>
       </c>
       <c r="C23" s="14">
         <f>C7*Inputs!$B$12*Inputs!$B$13</f>
-        <v/>
+        <v>87.45</v>
       </c>
       <c r="D23" s="14">
         <f>D7*Inputs!$B$12*Inputs!$B$13</f>
-        <v/>
+        <v>174.9</v>
       </c>
     </row>
     <row r="24">
@@ -1500,15 +1648,15 @@
       </c>
       <c r="B24" s="14">
         <f>Inputs!$B$14*Inputs!$B$15*12+Inputs!$B$16</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="C24" s="14">
         <f>Inputs!$B$14*Inputs!$B$15*12+Inputs!$B$16</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="D24" s="14">
         <f>Inputs!$B$14*Inputs!$B$15*12+Inputs!$B$16</f>
-        <v/>
+        <v>600</v>
       </c>
     </row>
     <row r="25">
@@ -1519,15 +1667,15 @@
       </c>
       <c r="B25" s="14">
         <f>Inputs!$B$17*12</f>
-        <v/>
+        <v>360</v>
       </c>
       <c r="C25" s="14">
         <f>Inputs!$B$17*12</f>
-        <v/>
+        <v>360</v>
       </c>
       <c r="D25" s="14">
         <f>Inputs!$B$17*12</f>
-        <v/>
+        <v>360</v>
       </c>
     </row>
     <row r="26">
@@ -1538,15 +1686,15 @@
       </c>
       <c r="B26" s="14">
         <f>B8*Inputs!$B$18*52</f>
-        <v/>
+        <v>14736.8</v>
       </c>
       <c r="C26" s="14">
         <f>C8*Inputs!$B$18*52</f>
-        <v/>
+        <v>14736.8</v>
       </c>
       <c r="D26" s="14">
         <f>D8*Inputs!$B$18*52</f>
-        <v/>
+        <v>22105.2</v>
       </c>
     </row>
     <row r="27">
@@ -1557,15 +1705,15 @@
       </c>
       <c r="B27" s="14">
         <f>B9*Inputs!$B$19*Inputs!$B$20</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C27" s="14">
         <f>C9*Inputs!$B$19*Inputs!$B$20</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D27" s="14">
         <f>D9*Inputs!$B$19*Inputs!$B$20</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1576,15 +1724,15 @@
       </c>
       <c r="B28" s="14">
         <f>B10</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C28" s="14">
         <f>C10</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D28" s="14">
         <f>D10</f>
-        <v/>
+        <v>24000</v>
       </c>
     </row>
     <row r="29">
@@ -1595,7 +1743,7 @@
       </c>
       <c r="B29" s="24">
         <f>Inputs!$B$21</f>
-        <v/>
+        <v>12000</v>
       </c>
       <c r="C29" s="18" t="n">
         <v>0</v>
@@ -1612,7 +1760,7 @@
       </c>
       <c r="B30" s="24">
         <f>Inputs!$B$22</f>
-        <v/>
+        <v>10000</v>
       </c>
       <c r="C30" s="18" t="n">
         <v>0</v>
@@ -1629,15 +1777,15 @@
       </c>
       <c r="B31" s="14">
         <f>B5*Inputs!$B$23</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="C31" s="14">
         <f>C5*Inputs!$B$23</f>
-        <v/>
+        <v>1000</v>
       </c>
       <c r="D31" s="14">
         <f>D5*Inputs!$B$23</f>
-        <v/>
+        <v>1600</v>
       </c>
     </row>
     <row r="32">
@@ -1664,15 +1812,15 @@
       </c>
       <c r="B33" s="13">
         <f>SUM(B21:B32)</f>
-        <v/>
+        <v>42361.87</v>
       </c>
       <c r="C33" s="13">
         <f>SUM(C21:C32)</f>
-        <v/>
+        <v>21417.85</v>
       </c>
       <c r="D33" s="13">
         <f>SUM(D21:D32)</f>
-        <v/>
+        <v>54515.7</v>
       </c>
     </row>
     <row r="35">
@@ -1683,15 +1831,15 @@
       </c>
       <c r="B35" s="13">
         <f>B18-B33</f>
-        <v/>
+        <v>-39661.87</v>
       </c>
       <c r="C35" s="13">
         <f>C18-C33</f>
-        <v/>
+        <v>-13417.85</v>
       </c>
       <c r="D35" s="13">
         <f>D18-D33</f>
-        <v/>
+        <v>-34715.7</v>
       </c>
     </row>
     <row r="36">
@@ -1702,15 +1850,15 @@
       </c>
       <c r="B36" s="13">
         <f>B35</f>
-        <v/>
+        <v>-39661.87</v>
       </c>
       <c r="C36" s="13">
         <f>B36+C35</f>
-        <v/>
+        <v>-53079.72</v>
       </c>
       <c r="D36" s="13">
         <f>C36+D35</f>
-        <v/>
+        <v>-87795.42</v>
       </c>
     </row>
     <row r="38">
@@ -1721,15 +1869,15 @@
       </c>
       <c r="B38" s="25">
         <f>IF(B4=0,0,B18/B4)</f>
-        <v/>
+        <v>18</v>
       </c>
       <c r="C38" s="25">
         <f>IF(C4=0,0,C18/C4)</f>
-        <v/>
+        <v>20</v>
       </c>
       <c r="D38" s="25">
         <f>IF(D4=0,0,D18/D4)</f>
-        <v/>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1910,15 +2058,15 @@
       </c>
       <c r="B13" s="14">
         <f>B4*Inputs!$B$3*12</f>
-        <v/>
+        <v>48000</v>
       </c>
       <c r="C13" s="14">
         <f>C4*Inputs!$B$3*12</f>
-        <v/>
+        <v>180000</v>
       </c>
       <c r="D13" s="14">
         <f>D4*Inputs!$B$3*12</f>
-        <v/>
+        <v>540000</v>
       </c>
     </row>
     <row r="14">
@@ -1929,15 +2077,15 @@
       </c>
       <c r="B14" s="14">
         <f>B4*B6</f>
-        <v/>
+        <v>40000</v>
       </c>
       <c r="C14" s="14">
         <f>C4*C6</f>
-        <v/>
+        <v>210000</v>
       </c>
       <c r="D14" s="14">
         <f>D4*D6</f>
-        <v/>
+        <v>810000</v>
       </c>
     </row>
     <row r="15">
@@ -1948,15 +2096,15 @@
       </c>
       <c r="B15" s="13">
         <f>B13+B14</f>
-        <v/>
+        <v>88000</v>
       </c>
       <c r="C15" s="13">
         <f>C13+C14</f>
-        <v/>
+        <v>390000</v>
       </c>
       <c r="D15" s="13">
         <f>D13+D14</f>
-        <v/>
+        <v>1350000</v>
       </c>
     </row>
     <row r="16">
@@ -1967,15 +2115,15 @@
       </c>
       <c r="B16" s="14">
         <f>B15*Inputs!$B$4</f>
-        <v/>
+        <v>8800</v>
       </c>
       <c r="C16" s="14">
         <f>C15*Inputs!$B$4</f>
-        <v/>
+        <v>39000</v>
       </c>
       <c r="D16" s="14">
         <f>D15*Inputs!$B$4</f>
-        <v/>
+        <v>135000</v>
       </c>
     </row>
     <row r="17">
@@ -1986,15 +2134,15 @@
       </c>
       <c r="B17" s="14">
         <f>Inputs!$B$9*((B13*(Inputs!$B$5+Inputs!$B$7))+(B4*12*Inputs!$B$6)+(B14*(Inputs!$B$5+Inputs!$B$7))+(B14/Inputs!$B$8*Inputs!$B$6))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C17" s="14">
         <f>Inputs!$B$9*((C13*(Inputs!$B$5+Inputs!$B$7))+(C4*12*Inputs!$B$6)+(C14*(Inputs!$B$5+Inputs!$B$7))+(C14/Inputs!$B$8*Inputs!$B$6))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D17" s="14">
         <f>Inputs!$B$9*((D13*(Inputs!$B$5+Inputs!$B$7))+(D4*12*Inputs!$B$6)+(D14*(Inputs!$B$5+Inputs!$B$7))+(D14/Inputs!$B$8*Inputs!$B$6))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -2005,15 +2153,15 @@
       </c>
       <c r="B18" s="13">
         <f>B16-B17</f>
-        <v/>
+        <v>8800</v>
       </c>
       <c r="C18" s="13">
         <f>C16-C17</f>
-        <v/>
+        <v>39000</v>
       </c>
       <c r="D18" s="13">
         <f>D16-D17</f>
-        <v/>
+        <v>135000</v>
       </c>
     </row>
     <row r="20">
@@ -2047,15 +2195,15 @@
       </c>
       <c r="B22" s="14">
         <f>B4*Inputs!$B$10*12/1000*Inputs!$B$11</f>
-        <v/>
+        <v>33.6</v>
       </c>
       <c r="C22" s="14">
         <f>C4*Inputs!$B$10*12/1000*Inputs!$B$11</f>
-        <v/>
+        <v>126</v>
       </c>
       <c r="D22" s="14">
         <f>D4*Inputs!$B$10*12/1000*Inputs!$B$11</f>
-        <v/>
+        <v>378</v>
       </c>
     </row>
     <row r="23">
@@ -2066,15 +2214,15 @@
       </c>
       <c r="B23" s="14">
         <f>B7*Inputs!$B$12*Inputs!$B$13</f>
-        <v/>
+        <v>139.92</v>
       </c>
       <c r="C23" s="14">
         <f>C7*Inputs!$B$12*Inputs!$B$13</f>
-        <v/>
+        <v>384.78</v>
       </c>
       <c r="D23" s="14">
         <f>D7*Inputs!$B$12*Inputs!$B$13</f>
-        <v/>
+        <v>874.5</v>
       </c>
     </row>
     <row r="24">
@@ -2085,15 +2233,15 @@
       </c>
       <c r="B24" s="14">
         <f>Inputs!$B$14*Inputs!$B$15*12+Inputs!$B$16</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="C24" s="14">
         <f>Inputs!$B$14*Inputs!$B$15*12+Inputs!$B$16</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="D24" s="14">
         <f>Inputs!$B$14*Inputs!$B$15*12+Inputs!$B$16</f>
-        <v/>
+        <v>600</v>
       </c>
     </row>
     <row r="25">
@@ -2104,15 +2252,15 @@
       </c>
       <c r="B25" s="14">
         <f>Inputs!$B$17*12</f>
-        <v/>
+        <v>360</v>
       </c>
       <c r="C25" s="14">
         <f>Inputs!$B$17*12</f>
-        <v/>
+        <v>360</v>
       </c>
       <c r="D25" s="14">
         <f>Inputs!$B$17*12</f>
-        <v/>
+        <v>360</v>
       </c>
     </row>
     <row r="26">
@@ -2123,15 +2271,15 @@
       </c>
       <c r="B26" s="14">
         <f>B8*Inputs!$B$18*52</f>
-        <v/>
+        <v>22105.2</v>
       </c>
       <c r="C26" s="14">
         <f>C8*Inputs!$B$18*52</f>
-        <v/>
+        <v>14736.8</v>
       </c>
       <c r="D26" s="14">
         <f>D8*Inputs!$B$18*52</f>
-        <v/>
+        <v>14736.8</v>
       </c>
     </row>
     <row r="27">
@@ -2142,15 +2290,15 @@
       </c>
       <c r="B27" s="14">
         <f>B9*Inputs!$B$19*Inputs!$B$20</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C27" s="14">
         <f>C9*Inputs!$B$19*Inputs!$B$20</f>
-        <v/>
+        <v>82500</v>
       </c>
       <c r="D27" s="14">
         <f>D9*Inputs!$B$19*Inputs!$B$20</f>
-        <v/>
+        <v>165000</v>
       </c>
     </row>
     <row r="28">
@@ -2161,15 +2309,15 @@
       </c>
       <c r="B28" s="14">
         <f>B10</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C28" s="14">
         <f>C10</f>
-        <v/>
+        <v>48000</v>
       </c>
       <c r="D28" s="14">
         <f>D10</f>
-        <v/>
+        <v>72000</v>
       </c>
     </row>
     <row r="29">
@@ -2180,7 +2328,7 @@
       </c>
       <c r="B29" s="24">
         <f>Inputs!$B$21</f>
-        <v/>
+        <v>12000</v>
       </c>
       <c r="C29" s="18" t="n">
         <v>6000</v>
@@ -2197,7 +2345,7 @@
       </c>
       <c r="B30" s="24">
         <f>Inputs!$B$22</f>
-        <v/>
+        <v>10000</v>
       </c>
       <c r="C30" s="18" t="n">
         <v>5000</v>
@@ -2214,15 +2362,15 @@
       </c>
       <c r="B31" s="14">
         <f>B5*Inputs!$B$23</f>
-        <v/>
+        <v>1200</v>
       </c>
       <c r="C31" s="14">
         <f>C5*Inputs!$B$23</f>
-        <v/>
+        <v>2400</v>
       </c>
       <c r="D31" s="14">
         <f>D5*Inputs!$B$23</f>
-        <v/>
+        <v>4000</v>
       </c>
     </row>
     <row r="32">
@@ -2249,15 +2397,15 @@
       </c>
       <c r="B33" s="13">
         <f>SUM(B21:B32)</f>
-        <v/>
+        <v>52038.72</v>
       </c>
       <c r="C33" s="13">
         <f>SUM(C21:C32)</f>
-        <v/>
+        <v>168707.58</v>
       </c>
       <c r="D33" s="13">
         <f>SUM(D21:D32)</f>
-        <v/>
+        <v>282749.3</v>
       </c>
     </row>
     <row r="35">
@@ -2268,15 +2416,15 @@
       </c>
       <c r="B35" s="13">
         <f>B18-B33</f>
-        <v/>
+        <v>-43238.72</v>
       </c>
       <c r="C35" s="13">
         <f>C18-C33</f>
-        <v/>
+        <v>-129707.58</v>
       </c>
       <c r="D35" s="13">
         <f>D18-D33</f>
-        <v/>
+        <v>-147749.3</v>
       </c>
     </row>
     <row r="36">
@@ -2287,15 +2435,15 @@
       </c>
       <c r="B36" s="13">
         <f>B35</f>
-        <v/>
+        <v>-43238.72</v>
       </c>
       <c r="C36" s="13">
         <f>B36+C35</f>
-        <v/>
+        <v>-172946.3</v>
       </c>
       <c r="D36" s="13">
         <f>C36+D35</f>
-        <v/>
+        <v>-320695.6</v>
       </c>
     </row>
     <row r="38">
@@ -2306,15 +2454,15 @@
       </c>
       <c r="B38" s="25">
         <f>IF(B4=0,0,B18/B4)</f>
-        <v/>
+        <v>22</v>
       </c>
       <c r="C38" s="25">
         <f>IF(C4=0,0,C18/C4)</f>
-        <v/>
+        <v>26</v>
       </c>
       <c r="D38" s="25">
         <f>IF(D4=0,0,D18/D4)</f>
-        <v/>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -2495,15 +2643,15 @@
       </c>
       <c r="B13" s="14">
         <f>B4*Inputs!$B$3*12</f>
-        <v/>
+        <v>120000</v>
       </c>
       <c r="C13" s="14">
         <f>C4*Inputs!$B$3*12</f>
-        <v/>
+        <v>600000</v>
       </c>
       <c r="D13" s="14">
         <f>D4*Inputs!$B$3*12</f>
-        <v/>
+        <v>1800000</v>
       </c>
     </row>
     <row r="14">
@@ -2514,15 +2662,15 @@
       </c>
       <c r="B14" s="14">
         <f>B4*B6</f>
-        <v/>
+        <v>150000</v>
       </c>
       <c r="C14" s="14">
         <f>C4*C6</f>
-        <v/>
+        <v>1100000</v>
       </c>
       <c r="D14" s="14">
         <f>D4*D6</f>
-        <v/>
+        <v>4500000</v>
       </c>
     </row>
     <row r="15">
@@ -2533,15 +2681,15 @@
       </c>
       <c r="B15" s="13">
         <f>B13+B14</f>
-        <v/>
+        <v>270000</v>
       </c>
       <c r="C15" s="13">
         <f>C13+C14</f>
-        <v/>
+        <v>1700000</v>
       </c>
       <c r="D15" s="13">
         <f>D13+D14</f>
-        <v/>
+        <v>6300000</v>
       </c>
     </row>
     <row r="16">
@@ -2552,15 +2700,15 @@
       </c>
       <c r="B16" s="14">
         <f>B15*Inputs!$B$4</f>
-        <v/>
+        <v>27000</v>
       </c>
       <c r="C16" s="14">
         <f>C15*Inputs!$B$4</f>
-        <v/>
+        <v>170000</v>
       </c>
       <c r="D16" s="14">
         <f>D15*Inputs!$B$4</f>
-        <v/>
+        <v>630000</v>
       </c>
     </row>
     <row r="17">
@@ -2571,15 +2719,15 @@
       </c>
       <c r="B17" s="14">
         <f>Inputs!$B$9*((B13*(Inputs!$B$5+Inputs!$B$7))+(B4*12*Inputs!$B$6)+(B14*(Inputs!$B$5+Inputs!$B$7))+(B14/Inputs!$B$8*Inputs!$B$6))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="C17" s="14">
         <f>Inputs!$B$9*((C13*(Inputs!$B$5+Inputs!$B$7))+(C4*12*Inputs!$B$6)+(C14*(Inputs!$B$5+Inputs!$B$7))+(C14/Inputs!$B$8*Inputs!$B$6))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D17" s="14">
         <f>Inputs!$B$9*((D13*(Inputs!$B$5+Inputs!$B$7))+(D4*12*Inputs!$B$6)+(D14*(Inputs!$B$5+Inputs!$B$7))+(D14/Inputs!$B$8*Inputs!$B$6))</f>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -2590,15 +2738,15 @@
       </c>
       <c r="B18" s="13">
         <f>B16-B17</f>
-        <v/>
+        <v>27000</v>
       </c>
       <c r="C18" s="13">
         <f>C16-C17</f>
-        <v/>
+        <v>170000</v>
       </c>
       <c r="D18" s="13">
         <f>D16-D17</f>
-        <v/>
+        <v>630000</v>
       </c>
     </row>
     <row r="20">
@@ -2632,15 +2780,15 @@
       </c>
       <c r="B22" s="14">
         <f>B4*Inputs!$B$10*12/1000*Inputs!$B$11</f>
-        <v/>
+        <v>84</v>
       </c>
       <c r="C22" s="14">
         <f>C4*Inputs!$B$10*12/1000*Inputs!$B$11</f>
-        <v/>
+        <v>420</v>
       </c>
       <c r="D22" s="14">
         <f>D4*Inputs!$B$10*12/1000*Inputs!$B$11</f>
-        <v/>
+        <v>1260</v>
       </c>
     </row>
     <row r="23">
@@ -2651,15 +2799,15 @@
       </c>
       <c r="B23" s="14">
         <f>B7*Inputs!$B$12*Inputs!$B$13</f>
-        <v/>
+        <v>349.8</v>
       </c>
       <c r="C23" s="14">
         <f>C7*Inputs!$B$12*Inputs!$B$13</f>
-        <v/>
+        <v>1224.3</v>
       </c>
       <c r="D23" s="14">
         <f>D7*Inputs!$B$12*Inputs!$B$13</f>
-        <v/>
+        <v>3148.2</v>
       </c>
     </row>
     <row r="24">
@@ -2670,15 +2818,15 @@
       </c>
       <c r="B24" s="14">
         <f>Inputs!$B$14*Inputs!$B$15*12+Inputs!$B$16</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="C24" s="14">
         <f>Inputs!$B$14*Inputs!$B$15*12+Inputs!$B$16</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="D24" s="14">
         <f>Inputs!$B$14*Inputs!$B$15*12+Inputs!$B$16</f>
-        <v/>
+        <v>600</v>
       </c>
     </row>
     <row r="25">
@@ -2689,15 +2837,15 @@
       </c>
       <c r="B25" s="14">
         <f>Inputs!$B$17*12</f>
-        <v/>
+        <v>360</v>
       </c>
       <c r="C25" s="14">
         <f>Inputs!$B$17*12</f>
-        <v/>
+        <v>360</v>
       </c>
       <c r="D25" s="14">
         <f>Inputs!$B$17*12</f>
-        <v/>
+        <v>360</v>
       </c>
     </row>
     <row r="26">
@@ -2708,15 +2856,15 @@
       </c>
       <c r="B26" s="14">
         <f>B8*Inputs!$B$18*52</f>
-        <v/>
+        <v>29473.6</v>
       </c>
       <c r="C26" s="14">
         <f>C8*Inputs!$B$18*52</f>
-        <v/>
+        <v>14736.8</v>
       </c>
       <c r="D26" s="14">
         <f>D8*Inputs!$B$18*52</f>
-        <v/>
+        <v>29473.6</v>
       </c>
     </row>
     <row r="27">
@@ -2727,15 +2875,15 @@
       </c>
       <c r="B27" s="14">
         <f>B9*Inputs!$B$19*Inputs!$B$20</f>
-        <v/>
+        <v>82500</v>
       </c>
       <c r="C27" s="14">
         <f>C9*Inputs!$B$19*Inputs!$B$20</f>
-        <v/>
+        <v>165000</v>
       </c>
       <c r="D27" s="14">
         <f>D9*Inputs!$B$19*Inputs!$B$20</f>
-        <v/>
+        <v>330000</v>
       </c>
     </row>
     <row r="28">
@@ -2746,15 +2894,15 @@
       </c>
       <c r="B28" s="14">
         <f>B10</f>
-        <v/>
+        <v>48000</v>
       </c>
       <c r="C28" s="14">
         <f>C10</f>
-        <v/>
+        <v>72000</v>
       </c>
       <c r="D28" s="14">
         <f>D10</f>
-        <v/>
+        <v>96000</v>
       </c>
     </row>
     <row r="29">
@@ -2765,7 +2913,7 @@
       </c>
       <c r="B29" s="24">
         <f>Inputs!$B$21</f>
-        <v/>
+        <v>12000</v>
       </c>
       <c r="C29" s="18" t="n">
         <v>12000</v>
@@ -2782,7 +2930,7 @@
       </c>
       <c r="B30" s="24">
         <f>Inputs!$B$22</f>
-        <v/>
+        <v>10000</v>
       </c>
       <c r="C30" s="18" t="n">
         <v>10000</v>
@@ -2799,15 +2947,15 @@
       </c>
       <c r="B31" s="14">
         <f>B5*Inputs!$B$23</f>
-        <v/>
+        <v>2000</v>
       </c>
       <c r="C31" s="14">
         <f>C5*Inputs!$B$23</f>
-        <v/>
+        <v>5000</v>
       </c>
       <c r="D31" s="14">
         <f>D5*Inputs!$B$23</f>
-        <v/>
+        <v>10000</v>
       </c>
     </row>
     <row r="32">
@@ -2834,15 +2982,15 @@
       </c>
       <c r="B33" s="13">
         <f>SUM(B21:B32)</f>
-        <v/>
+        <v>193967.4</v>
       </c>
       <c r="C33" s="13">
         <f>SUM(C21:C32)</f>
-        <v/>
+        <v>302341.1</v>
       </c>
       <c r="D33" s="13">
         <f>SUM(D21:D32)</f>
-        <v/>
+        <v>523841.8</v>
       </c>
     </row>
     <row r="35">
@@ -2853,15 +3001,15 @@
       </c>
       <c r="B35" s="13">
         <f>B18-B33</f>
-        <v/>
+        <v>-166967.4</v>
       </c>
       <c r="C35" s="13">
         <f>C18-C33</f>
-        <v/>
+        <v>-132341.1</v>
       </c>
       <c r="D35" s="13">
         <f>D18-D33</f>
-        <v/>
+        <v>106158.2</v>
       </c>
     </row>
     <row r="36">
@@ -2872,15 +3020,15 @@
       </c>
       <c r="B36" s="13">
         <f>B35</f>
-        <v/>
+        <v>-166967.4</v>
       </c>
       <c r="C36" s="13">
         <f>B36+C35</f>
-        <v/>
+        <v>-299308.5</v>
       </c>
       <c r="D36" s="13">
         <f>C36+D35</f>
-        <v/>
+        <v>-193150.3</v>
       </c>
     </row>
     <row r="38">
@@ -2891,15 +3039,15 @@
       </c>
       <c r="B38" s="25">
         <f>IF(B4=0,0,B18/B4)</f>
-        <v/>
+        <v>27</v>
       </c>
       <c r="C38" s="25">
         <f>IF(C4=0,0,C18/C4)</f>
-        <v/>
+        <v>34</v>
       </c>
       <c r="D38" s="25">
         <f>IF(D4=0,0,D18/D4)</f>
-        <v/>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -2954,15 +3102,15 @@
       </c>
       <c r="B3" s="26">
         <f>S!D4</f>
-        <v/>
+        <v>900</v>
       </c>
       <c r="C3" s="26">
         <f>M!D4</f>
-        <v/>
+        <v>4500</v>
       </c>
       <c r="D3" s="26">
         <f>L!D4</f>
-        <v/>
+        <v>15000</v>
       </c>
     </row>
     <row r="4">
@@ -2973,15 +3121,15 @@
       </c>
       <c r="B4" s="24">
         <f>S!D15</f>
-        <v/>
+        <v>198000</v>
       </c>
       <c r="C4" s="24">
         <f>M!D15</f>
-        <v/>
+        <v>1350000</v>
       </c>
       <c r="D4" s="24">
         <f>L!D15</f>
-        <v/>
+        <v>6300000</v>
       </c>
     </row>
     <row r="5">
@@ -2992,15 +3140,15 @@
       </c>
       <c r="B5" s="24">
         <f>S!D18</f>
-        <v/>
+        <v>19800</v>
       </c>
       <c r="C5" s="24">
         <f>M!D18</f>
-        <v/>
+        <v>135000</v>
       </c>
       <c r="D5" s="24">
         <f>L!D18</f>
-        <v/>
+        <v>630000</v>
       </c>
     </row>
     <row r="6">
@@ -3011,15 +3159,15 @@
       </c>
       <c r="B6" s="24">
         <f>S!D33</f>
-        <v/>
+        <v>54515.7</v>
       </c>
       <c r="C6" s="24">
         <f>M!D33</f>
-        <v/>
+        <v>282749.3</v>
       </c>
       <c r="D6" s="24">
         <f>L!D33</f>
-        <v/>
+        <v>523841.8</v>
       </c>
     </row>
     <row r="7">
@@ -3030,15 +3178,15 @@
       </c>
       <c r="B7" s="24">
         <f>S!D35</f>
-        <v/>
+        <v>-34715.7</v>
       </c>
       <c r="C7" s="24">
         <f>M!D35</f>
-        <v/>
+        <v>-147749.3</v>
       </c>
       <c r="D7" s="24">
         <f>L!D35</f>
-        <v/>
+        <v>106158.2</v>
       </c>
     </row>
     <row r="8">
@@ -3049,15 +3197,15 @@
       </c>
       <c r="B8" s="24">
         <f>S!D36</f>
-        <v/>
+        <v>-87795.42</v>
       </c>
       <c r="C8" s="24">
         <f>M!D36</f>
-        <v/>
+        <v>-320695.6</v>
       </c>
       <c r="D8" s="24">
         <f>L!D36</f>
-        <v/>
+        <v>-193150.3</v>
       </c>
     </row>
     <row r="10">
@@ -3068,7 +3216,7 @@
       </c>
       <c r="B10" s="24">
         <f>'Sweat Equity'!B13</f>
-        <v/>
+        <v>38762.5</v>
       </c>
     </row>
     <row r="12">

</xml_diff>